<commit_message>
Integrate weekly game events
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.playerAttribute.xlsx
+++ b/Config/Luban/Datas/#game.playerAttribute.xlsx
@@ -802,7 +802,7 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>程序房间1点行动属性获得量</t>
+          <t>程序房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -810,7 +810,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>进入程序房间触发选项时，选择消耗1点行动点获得的属性数值</t>
+          <t>进入程序房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -821,7 +821,7 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>程序房间2点行动属性获得量</t>
+          <t>程序房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -829,7 +829,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>进入程序房间触发选项时，选择消耗2点行动点获得的属性数值</t>
+          <t>进入程序房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>程序房间每行动点属性获得量</t>
+          <t>程序房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -848,7 +848,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>每在程序房间消耗1点行动点额外获得的属性数值</t>
+          <t>每在程序房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>美术房间1点行动属性获得量</t>
+          <t>美术房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -867,7 +867,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>进入美术房间触发选项时，选择消耗1点行动点获得的属性数值</t>
+          <t>进入美术房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -878,7 +878,7 @@
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>美术房间2点行动属性获得量</t>
+          <t>美术房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -886,7 +886,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>进入美术房间触发选项时，选择消耗2点行动点获得的属性数值</t>
+          <t>进入美术房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -897,7 +897,7 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>美术房间每行动点属性获得量</t>
+          <t>美术房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -905,7 +905,7 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>每在美术房间消耗1点行动点额外获得的属性数值</t>
+          <t>每在美术房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>音效房间1点行动属性获得量</t>
+          <t>音效房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -924,7 +924,7 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>进入音效房间触发选项时，选择消耗1点行动点获得的属性数值</t>
+          <t>进入音效房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -935,7 +935,7 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>音效房间2点行动属性获得量</t>
+          <t>音效房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -943,7 +943,7 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>进入音效房间触发选项时，选择消耗2点行动点获得的属性数值</t>
+          <t>进入音效房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
@@ -954,7 +954,7 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>音效房间每行动点属性获得量</t>
+          <t>音效房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -962,7 +962,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>每在音效房间消耗1点行动点额外获得的属性数值</t>
+          <t>每在音效房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update event config and month settlement
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.playerAttribute.xlsx
+++ b/Config/Luban/Datas/#game.playerAttribute.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E44"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -589,144 +589,144 @@
     <row r="7" ht="28" customHeight="1">
       <c r="A7" s="3" t="n"/>
       <c r="B7" s="3" t="n">
-        <v>1003</v>
+        <v>1043</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>月发金币</t>
+          <t>程序房间基础周操作次数</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1000</v>
+        <v>1</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>每个月开始时发放的金币</t>
+          <t>每周刷新程序房间可操作次数时使用的基础值</t>
         </is>
       </c>
     </row>
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="3" t="n"/>
       <c r="B8" s="3" t="n">
-        <v>1008</v>
+        <v>1044</v>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>金币</t>
+          <t>程序房间周操作次数</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>当前持有金币，唯一货币</t>
+          <t>当前周程序房间剩余可操作次数，操作会消耗</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="n"/>
       <c r="B9" s="3" t="n">
-        <v>1009</v>
+        <v>1045</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>愿望单数量</t>
+          <t>美术房间基础周操作次数</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>当前愿望单数量</t>
+          <t>每周刷新美术房间可操作次数时使用的基础值</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="3" t="n">
-        <v>1004</v>
+        <v>1046</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>周愿望增长</t>
+          <t>美术房间周操作次数</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>每周结算时的基础愿望单增长</t>
+          <t>当前周美术房间剩余可操作次数，操作会消耗</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="3" t="n">
-        <v>1005</v>
+        <v>1047</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Bug 值</t>
+          <t>音效房间基础周操作次数</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>当前Bug值</t>
+          <t>每周刷新音效房间可操作次数时使用的基础值</t>
         </is>
       </c>
     </row>
     <row r="12" ht="28" customHeight="1">
       <c r="A12" s="3" t="n"/>
       <c r="B12" s="3" t="n">
-        <v>1006</v>
+        <v>1048</v>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>画面</t>
+          <t>音效房间周操作次数</t>
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>画面表现分</t>
+          <t>当前周音效房间剩余可操作次数，操作会消耗</t>
         </is>
       </c>
     </row>
     <row r="13" ht="28" customHeight="1">
       <c r="A13" s="3" t="n"/>
       <c r="B13" s="3" t="n">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>氛围</t>
+          <t>月发金币</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>氛围表现分</t>
+          <t>每个月开始时发放的金币</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="n"/>
       <c r="B14" s="3" t="n">
-        <v>1028</v>
+        <v>1008</v>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>每周Bug值变化</t>
+          <t>金币</t>
         </is>
       </c>
       <c r="D14" s="3" t="n">
@@ -734,18 +734,18 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>每周结算时应用的Bug值变化量</t>
+          <t>当前持有金币，唯一货币</t>
         </is>
       </c>
     </row>
     <row r="15" ht="70" customHeight="1">
       <c r="A15" s="3" t="n"/>
       <c r="B15" s="3" t="n">
-        <v>1029</v>
+        <v>1009</v>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>每周画面值变化</t>
+          <t>愿望单数量</t>
         </is>
       </c>
       <c r="D15" s="3" t="n">
@@ -753,37 +753,37 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>每周结算时应用的画面值变化量</t>
+          <t>当前愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="16" ht="70" customHeight="1">
       <c r="A16" s="3" t="n"/>
       <c r="B16" s="3" t="n">
-        <v>1030</v>
+        <v>1004</v>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>每周氛围值变化</t>
+          <t>周愿望增长</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>每周结算时应用的氛围值变化量</t>
+          <t>每周结算时的基础愿望单增长</t>
         </is>
       </c>
     </row>
     <row r="17" ht="70" customHeight="1">
       <c r="A17" s="3" t="n"/>
       <c r="B17" s="3" t="n">
-        <v>1011</v>
+        <v>1005</v>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>程序房间1AP愿望单获得量</t>
+          <t>Bug 值</t>
         </is>
       </c>
       <c r="D17" s="3" t="n">
@@ -791,18 +791,18 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>进入程序房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+          <t>当前Bug值</t>
         </is>
       </c>
     </row>
     <row r="18" ht="70" customHeight="1">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="3" t="n">
-        <v>1012</v>
+        <v>1006</v>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>程序房间2AP愿望单获得量</t>
+          <t>画面</t>
         </is>
       </c>
       <c r="D18" s="3" t="n">
@@ -810,18 +810,18 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>进入程序房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+          <t>画面表现分</t>
         </is>
       </c>
     </row>
     <row r="19" ht="70" customHeight="1">
       <c r="A19" s="3" t="n"/>
       <c r="B19" s="3" t="n">
-        <v>1017</v>
+        <v>1007</v>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>程序房间每AP愿望单获得量</t>
+          <t>氛围</t>
         </is>
       </c>
       <c r="D19" s="3" t="n">
@@ -829,18 +829,18 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>每在程序房间消耗1点行动点额外获得的愿望单数量</t>
+          <t>氛围表现分</t>
         </is>
       </c>
     </row>
     <row r="20" ht="70" customHeight="1">
       <c r="A20" s="3" t="n"/>
       <c r="B20" s="3" t="n">
-        <v>1013</v>
+        <v>1028</v>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>美术房间1AP愿望单获得量</t>
+          <t>每周Bug值变化</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
@@ -848,18 +848,18 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>进入美术房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+          <t>每周结算时应用的Bug值变化量</t>
         </is>
       </c>
     </row>
     <row r="21" ht="56" customHeight="1">
       <c r="A21" s="3" t="n"/>
       <c r="B21" s="3" t="n">
-        <v>1014</v>
+        <v>1029</v>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>美术房间2AP愿望单获得量</t>
+          <t>每周画面值变化</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
@@ -867,18 +867,18 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>进入美术房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+          <t>每周结算时应用的画面值变化量</t>
         </is>
       </c>
     </row>
     <row r="22" ht="56" customHeight="1">
       <c r="A22" s="3" t="n"/>
       <c r="B22" s="3" t="n">
-        <v>1018</v>
+        <v>1030</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>美术房间每AP愿望单获得量</t>
+          <t>每周氛围值变化</t>
         </is>
       </c>
       <c r="D22" s="3" t="n">
@@ -886,18 +886,18 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>每在美术房间消耗1点行动点额外获得的愿望单数量</t>
+          <t>每周结算时应用的氛围值变化量</t>
         </is>
       </c>
     </row>
     <row r="23" ht="56" customHeight="1">
       <c r="A23" s="3" t="n"/>
       <c r="B23" s="3" t="n">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>音效房间1AP愿望单获得量</t>
+          <t>程序房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
@@ -905,18 +905,18 @@
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>进入音效房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+          <t>进入程序房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="24" ht="56" customHeight="1">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="3" t="n">
-        <v>1016</v>
+        <v>1012</v>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>音效房间2AP愿望单获得量</t>
+          <t>程序房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D24" s="3" t="n">
@@ -924,18 +924,18 @@
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>进入音效房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+          <t>进入程序房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="25" ht="56" customHeight="1">
       <c r="A25" s="3" t="n"/>
       <c r="B25" s="3" t="n">
-        <v>1019</v>
+        <v>1017</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>音效房间每AP愿望单获得量</t>
+          <t>程序房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D25" s="3" t="n">
@@ -943,18 +943,18 @@
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>每在音效房间消耗1点行动点额外获得的愿望单数量</t>
+          <t>每在程序房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="26" ht="42" customHeight="1">
       <c r="A26" s="3" t="n"/>
       <c r="B26" s="3" t="n">
-        <v>1020</v>
+        <v>1013</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>连续同房间行动愿望单奖励</t>
+          <t>美术房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D26" s="3" t="n">
@@ -962,18 +962,18 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>连续两回合在同一房间消耗行动点时获得的愿望单数量</t>
+          <t>进入美术房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="27" ht="42" customHeight="1">
       <c r="A27" s="3" t="n"/>
       <c r="B27" s="3" t="n">
-        <v>1021</v>
+        <v>1014</v>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>回合开始50%愿望单倍率</t>
+          <t>美术房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
@@ -981,18 +981,18 @@
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>每回合开始时，有50%概率获得的愿望单倍率</t>
+          <t>进入美术房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="28" ht="28" customHeight="1">
       <c r="A28" s="3" t="n"/>
       <c r="B28" s="3" t="n">
-        <v>1022</v>
+        <v>1018</v>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>3/6/9回合结束愿望单奖励</t>
+          <t>美术房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D28" s="3" t="n">
@@ -1000,18 +1000,18 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>第3、6、9回合结束时获得的愿望单数量</t>
+          <t>每在美术房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="29" ht="56" customHeight="1">
       <c r="A29" s="3" t="n"/>
       <c r="B29" s="3" t="n">
-        <v>1023</v>
+        <v>1015</v>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>低Bug每回合愿望单奖励</t>
+          <t>音效房间1AP愿望单获得量</t>
         </is>
       </c>
       <c r="D29" s="3" t="n">
@@ -1019,18 +1019,18 @@
       </c>
       <c r="E29" s="3" t="inlineStr">
         <is>
-          <t>Bug低于40时，每回合获得的愿望单数量</t>
+          <t>进入音效房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="30" ht="70" customHeight="1">
       <c r="A30" s="3" t="n"/>
       <c r="B30" s="3" t="n">
-        <v>1024</v>
+        <v>1016</v>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>愿望单增长百分比加成</t>
+          <t>音效房间2AP愿望单获得量</t>
         </is>
       </c>
       <c r="D30" s="3" t="n">
@@ -1038,18 +1038,18 @@
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>愿望单增长量提高百分比</t>
+          <t>进入音效房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="31" ht="84" customHeight="1">
       <c r="A31" s="3" t="n"/>
       <c r="B31" s="3" t="n">
-        <v>1025</v>
+        <v>1019</v>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>高画面回合结束愿望单增长加成</t>
+          <t>音效房间每AP愿望单获得量</t>
         </is>
       </c>
       <c r="D31" s="3" t="n">
@@ -1057,240 +1057,354 @@
       </c>
       <c r="E31" s="3" t="inlineStr">
         <is>
-          <t>每回合结束时画面值高于60时，愿望单增长量提高量</t>
+          <t>每在音效房间消耗1点行动点额外获得的愿望单数量</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="n"/>
       <c r="B32" s="3" t="n">
+        <v>1020</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>连续同房间行动愿望单奖励</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>连续两回合在同一房间消耗行动点时获得的愿望单数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="n"/>
+      <c r="B33" s="3" t="n">
+        <v>1021</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>回合开始50%愿望单倍率</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>每回合开始时，有50%概率获得的愿望单倍率</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="n"/>
+      <c r="B34" s="3" t="n">
+        <v>1022</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>3/6/9回合结束愿望单奖励</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>第3、6、9回合结束时获得的愿望单数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="3" t="n">
+        <v>1023</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>低Bug每回合愿望单奖励</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Bug低于40时，每回合获得的愿望单数量</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="n"/>
+      <c r="B36" s="3" t="n">
+        <v>1024</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>愿望单增长百分比加成</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>愿望单增长量提高百分比</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="3" t="n">
+        <v>1025</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>高画面回合结束愿望单增长加成</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>每回合结束时画面值高于60时，愿望单增长量提高量</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="n"/>
+      <c r="B38" s="3" t="n">
         <v>1026</v>
       </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>三房间同回合行动愿望单增长加成</t>
         </is>
       </c>
-      <c r="D32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="D38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
         <is>
           <t>同一回合在三个房间都消耗行动点时，愿望单增长量提高量</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="B33" t="n">
-        <v>1031</v>
-      </c>
-      <c r="C33" t="inlineStr">
-        <is>
-          <t>程序1AP Bug变化最小值</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>-4</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>程序房间消耗1点行动点时，Bug变化随机下限（负数表示降低）</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="B34" t="n">
-        <v>1032</v>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>程序1AP Bug变化最大值</t>
-        </is>
-      </c>
-      <c r="D34" t="n">
-        <v>-2</v>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>程序房间消耗1点行动点时，Bug变化随机上限（负数表示降低）</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="B35" t="n">
-        <v>1033</v>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>程序2AP Bug变化最小值</t>
-        </is>
-      </c>
-      <c r="D35" t="n">
-        <v>-9</v>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>程序房间消耗2点行动点时，Bug变化随机下限（负数表示降低）</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="B36" t="n">
-        <v>1034</v>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>程序2AP Bug变化最大值</t>
-        </is>
-      </c>
-      <c r="D36" t="n">
-        <v>-6</v>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>程序房间消耗2点行动点时，Bug变化随机上限（负数表示降低）</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="B37" t="n">
-        <v>1035</v>
-      </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>美术1AP画面变化最小值</t>
-        </is>
-      </c>
-      <c r="D37" t="n">
-        <v>5</v>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>美术房间消耗1点行动点时，画面变化随机下限</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="B38" t="n">
-        <v>1036</v>
-      </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>美术1AP画面变化最大值</t>
-        </is>
-      </c>
-      <c r="D38" t="n">
-        <v>7</v>
-      </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>美术房间消耗1点行动点时，画面变化随机上限</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="B39" t="n">
-        <v>1037</v>
+        <v>1031</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>美术2AP画面变化最小值</t>
+          <t>程序1AP Bug变化最小值</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>13</v>
+        <v>-4</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>美术房间消耗2点行动点时，画面变化随机下限</t>
+          <t>程序房间消耗1点行动点时，Bug变化随机下限（负数表示降低）</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="n">
-        <v>1038</v>
+        <v>1032</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>美术2AP画面变化最大值</t>
+          <t>程序1AP Bug变化最大值</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>15</v>
+        <v>-2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>美术房间消耗2点行动点时，画面变化随机上限</t>
+          <t>程序房间消耗1点行动点时，Bug变化随机上限（负数表示降低）</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="n">
-        <v>1039</v>
+        <v>1033</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>音效1AP氛围变化最小值</t>
+          <t>程序2AP Bug变化最小值</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>5</v>
+        <v>-9</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>音效房间消耗1点行动点时，氛围变化随机下限</t>
+          <t>程序房间消耗2点行动点时，Bug变化随机下限（负数表示降低）</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="B42" t="n">
-        <v>1040</v>
+        <v>1034</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>音效1AP氛围变化最大值</t>
+          <t>程序2AP Bug变化最大值</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>7</v>
+        <v>-6</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>音效房间消耗1点行动点时，氛围变化随机上限</t>
+          <t>程序房间消耗2点行动点时，Bug变化随机上限（负数表示降低）</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="n">
-        <v>1041</v>
+        <v>1035</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>音效2AP氛围变化最小值</t>
+          <t>美术1AP画面变化最小值</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>音效房间消耗2点行动点时，氛围变化随机下限</t>
+          <t>美术房间消耗1点行动点时，画面变化随机下限</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="n">
+        <v>1036</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>美术1AP画面变化最大值</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>7</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>美术房间消耗1点行动点时，画面变化随机上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="n">
+        <v>1037</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>美术2AP画面变化最小值</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>13</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>美术房间消耗2点行动点时，画面变化随机下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="n">
+        <v>1038</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>美术2AP画面变化最大值</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>15</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>美术房间消耗2点行动点时，画面变化随机上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" t="n">
+        <v>1039</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>音效1AP氛围变化最小值</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>5</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>音效房间消耗1点行动点时，氛围变化随机下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" t="n">
+        <v>1040</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>音效1AP氛围变化最大值</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>7</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>音效房间消耗1点行动点时，氛围变化随机上限</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" t="n">
+        <v>1041</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>音效2AP氛围变化最小值</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>12</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>音效房间消耗2点行动点时，氛围变化随机下限</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" t="n">
         <v>1042</v>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C50" t="inlineStr">
         <is>
           <t>音效2AP氛围变化最大值</t>
         </is>
       </c>
-      <c r="D44" t="n">
+      <c r="D50" t="n">
         <v>15</v>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E50" t="inlineStr">
         <is>
           <t>音效房间消耗2点行动点时，氛围变化随机上限</t>
         </is>

</xml_diff>

<commit_message>
Add budget shop purchase limits
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.playerAttribute.xlsx
+++ b/Config/Luban/Datas/#game.playerAttribute.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1410,6 +1410,42 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="B51" t="n">
+        <v>1049</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>每次商店购买次数</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>每次进入商店时可购买Buff的次数</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" t="n">
+        <v>1050</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>当前商店购买次数</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>0</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>当前商店阶段剩余可购买Buff的次数，进入商店时按每次商店购买次数重置</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add weekly flow attribute modifiers
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.playerAttribute.xlsx
+++ b/Config/Luban/Datas/#game.playerAttribute.xlsx
@@ -445,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E57"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1446,6 +1446,96 @@
         </is>
       </c>
     </row>
+    <row r="53">
+      <c r="B53" t="n">
+        <v>1051</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>当前月第几周</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>0</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>只读流程镜像；用于配表条件判断，表示当前月内第几周，不允许通过事件或Buff修改</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="B54" t="n">
+        <v>1052</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>全局第几周</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>0</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>只读流程镜像；用于配表条件判断，表示从开局累计到当前的第几周，不允许通过事件或Buff修改</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="B55" t="n">
+        <v>1053</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>本周程序AP额外Bug变化</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>0</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>本周每消耗1点程序AP时额外应用的Bug变化；进入下一周自动清零</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="B56" t="n">
+        <v>1054</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>本周美术AP额外画面变化</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>0</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>本周每消耗1点美术AP时额外应用的画面变化；进入下一周自动清零</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="B57" t="n">
+        <v>1055</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>本周音频AP额外氛围变化</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>0</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>本周每消耗1点音频AP时额外应用的氛围变化；进入下一周自动清零</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update player attribute config
</commit_message>
<xml_diff>
--- a/Config/Luban/Datas/#game.playerAttribute.xlsx
+++ b/Config/Luban/Datas/#game.playerAttribute.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\AXR_Projects\unity\Anchor\Config\Luban\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C91CADED-3080-412E-8F19-DAA8DD69ABF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B995DAE-5AB5-4ED5-BAC5-AA3DC6363298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,241 +145,242 @@
     <t>画面</t>
   </si>
   <si>
+    <t>氛围</t>
+  </si>
+  <si>
+    <t>氛围表现分</t>
+  </si>
+  <si>
+    <t>每周Bug值变化</t>
+  </si>
+  <si>
+    <t>每周结算时应用的Bug值变化量</t>
+  </si>
+  <si>
+    <t>每周画面值变化</t>
+  </si>
+  <si>
+    <t>每周结算时应用的画面值变化量</t>
+  </si>
+  <si>
+    <t>每周氛围值变化</t>
+  </si>
+  <si>
+    <t>每周结算时应用的氛围值变化量</t>
+  </si>
+  <si>
+    <t>程序房间1AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入程序房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>程序房间2AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入程序房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>程序房间每AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>每在程序房间消耗1点行动点额外获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>美术房间1AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入美术房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>美术房间2AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入美术房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>美术房间每AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>每在美术房间消耗1点行动点额外获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>音效房间1AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入音效房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>音效房间2AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>进入音效房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>音效房间每AP愿望单获得量</t>
+  </si>
+  <si>
+    <t>每在音效房间消耗1点行动点额外获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>连续同房间行动愿望单奖励</t>
+  </si>
+  <si>
+    <t>连续两回合在同一房间消耗行动点时获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>回合开始50%愿望单倍率</t>
+  </si>
+  <si>
+    <t>每回合开始时，有50%概率获得的愿望单倍率</t>
+  </si>
+  <si>
+    <t>3/6/9回合结束愿望单奖励</t>
+  </si>
+  <si>
+    <t>第3、6、9回合结束时获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>低Bug每回合愿望单奖励</t>
+  </si>
+  <si>
+    <t>Bug低于40时，每回合获得的愿望单数量</t>
+  </si>
+  <si>
+    <t>愿望单增长百分比加成</t>
+  </si>
+  <si>
+    <t>愿望单增长量提高百分比</t>
+  </si>
+  <si>
+    <t>高画面回合结束愿望单增长加成</t>
+  </si>
+  <si>
+    <t>每回合结束时画面值高于60时，愿望单增长量提高量</t>
+  </si>
+  <si>
+    <t>三房间同回合行动愿望单增长加成</t>
+  </si>
+  <si>
+    <t>同一回合在三个房间都消耗行动点时，愿望单增长量提高量</t>
+  </si>
+  <si>
+    <t>程序1AP Bug变化最小值</t>
+  </si>
+  <si>
+    <t>程序房间消耗1点行动点时，Bug变化随机下限（负数表示降低）</t>
+  </si>
+  <si>
+    <t>程序1AP Bug变化最大值</t>
+  </si>
+  <si>
+    <t>程序房间消耗1点行动点时，Bug变化随机上限（负数表示降低）</t>
+  </si>
+  <si>
+    <t>程序2AP Bug变化最小值</t>
+  </si>
+  <si>
+    <t>程序房间消耗2点行动点时，Bug变化随机下限（负数表示降低）</t>
+  </si>
+  <si>
+    <t>程序2AP Bug变化最大值</t>
+  </si>
+  <si>
+    <t>程序房间消耗2点行动点时，Bug变化随机上限（负数表示降低）</t>
+  </si>
+  <si>
+    <t>美术1AP画面变化最小值</t>
+  </si>
+  <si>
+    <t>美术房间消耗1点行动点时，画面变化随机下限</t>
+  </si>
+  <si>
+    <t>美术1AP画面变化最大值</t>
+  </si>
+  <si>
+    <t>美术房间消耗1点行动点时，画面变化随机上限</t>
+  </si>
+  <si>
+    <t>美术2AP画面变化最小值</t>
+  </si>
+  <si>
+    <t>美术房间消耗2点行动点时，画面变化随机下限</t>
+  </si>
+  <si>
+    <t>美术2AP画面变化最大值</t>
+  </si>
+  <si>
+    <t>美术房间消耗2点行动点时，画面变化随机上限</t>
+  </si>
+  <si>
+    <t>音效1AP氛围变化最小值</t>
+  </si>
+  <si>
+    <t>音效房间消耗1点行动点时，氛围变化随机下限</t>
+  </si>
+  <si>
+    <t>音效1AP氛围变化最大值</t>
+  </si>
+  <si>
+    <t>音效房间消耗1点行动点时，氛围变化随机上限</t>
+  </si>
+  <si>
+    <t>音效2AP氛围变化最小值</t>
+  </si>
+  <si>
+    <t>音效房间消耗2点行动点时，氛围变化随机下限</t>
+  </si>
+  <si>
+    <t>音效2AP氛围变化最大值</t>
+  </si>
+  <si>
+    <t>音效房间消耗2点行动点时，氛围变化随机上限</t>
+  </si>
+  <si>
+    <t>每次商店购买次数</t>
+  </si>
+  <si>
+    <t>每次进入商店时可购买Buff的次数</t>
+  </si>
+  <si>
+    <t>当前商店购买次数</t>
+  </si>
+  <si>
+    <t>当前商店阶段剩余可购买Buff的次数，进入商店时按每次商店购买次数重置</t>
+  </si>
+  <si>
+    <t>当前月第几周</t>
+  </si>
+  <si>
+    <t>只读流程镜像；用于配表条件判断，表示当前月内第几周，不允许通过事件或Buff修改</t>
+  </si>
+  <si>
+    <t>全局第几周</t>
+  </si>
+  <si>
+    <t>只读流程镜像；用于配表条件判断，表示从开局累计到当前的第几周，不允许通过事件或Buff修改</t>
+  </si>
+  <si>
+    <t>本周程序AP额外Bug变化</t>
+  </si>
+  <si>
+    <t>本周每消耗1点程序AP时额外应用的Bug变化；进入下一周自动清零</t>
+  </si>
+  <si>
+    <t>本周美术AP额外画面变化</t>
+  </si>
+  <si>
+    <t>本周每消耗1点美术AP时额外应用的画面变化；进入下一周自动清零</t>
+  </si>
+  <si>
+    <t>本周音频AP额外氛围变化</t>
+  </si>
+  <si>
+    <t>本周每消耗1点音频AP时额外应用的氛围变化；进入下一周自动清零</t>
+  </si>
+  <si>
     <t>画面表现分</t>
-  </si>
-  <si>
-    <t>氛围</t>
-  </si>
-  <si>
-    <t>氛围表现分</t>
-  </si>
-  <si>
-    <t>每周Bug值变化</t>
-  </si>
-  <si>
-    <t>每周结算时应用的Bug值变化量</t>
-  </si>
-  <si>
-    <t>每周画面值变化</t>
-  </si>
-  <si>
-    <t>每周结算时应用的画面值变化量</t>
-  </si>
-  <si>
-    <t>每周氛围值变化</t>
-  </si>
-  <si>
-    <t>每周结算时应用的氛围值变化量</t>
-  </si>
-  <si>
-    <t>程序房间1AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入程序房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>程序房间2AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入程序房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>程序房间每AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>每在程序房间消耗1点行动点额外获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>美术房间1AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入美术房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>美术房间2AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入美术房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>美术房间每AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>每在美术房间消耗1点行动点额外获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>音效房间1AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入音效房间触发选项时，选择消耗1点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>音效房间2AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>进入音效房间触发选项时，选择消耗2点行动点获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>音效房间每AP愿望单获得量</t>
-  </si>
-  <si>
-    <t>每在音效房间消耗1点行动点额外获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>连续同房间行动愿望单奖励</t>
-  </si>
-  <si>
-    <t>连续两回合在同一房间消耗行动点时获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>回合开始50%愿望单倍率</t>
-  </si>
-  <si>
-    <t>每回合开始时，有50%概率获得的愿望单倍率</t>
-  </si>
-  <si>
-    <t>3/6/9回合结束愿望单奖励</t>
-  </si>
-  <si>
-    <t>第3、6、9回合结束时获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>低Bug每回合愿望单奖励</t>
-  </si>
-  <si>
-    <t>Bug低于40时，每回合获得的愿望单数量</t>
-  </si>
-  <si>
-    <t>愿望单增长百分比加成</t>
-  </si>
-  <si>
-    <t>愿望单增长量提高百分比</t>
-  </si>
-  <si>
-    <t>高画面回合结束愿望单增长加成</t>
-  </si>
-  <si>
-    <t>每回合结束时画面值高于60时，愿望单增长量提高量</t>
-  </si>
-  <si>
-    <t>三房间同回合行动愿望单增长加成</t>
-  </si>
-  <si>
-    <t>同一回合在三个房间都消耗行动点时，愿望单增长量提高量</t>
-  </si>
-  <si>
-    <t>程序1AP Bug变化最小值</t>
-  </si>
-  <si>
-    <t>程序房间消耗1点行动点时，Bug变化随机下限（负数表示降低）</t>
-  </si>
-  <si>
-    <t>程序1AP Bug变化最大值</t>
-  </si>
-  <si>
-    <t>程序房间消耗1点行动点时，Bug变化随机上限（负数表示降低）</t>
-  </si>
-  <si>
-    <t>程序2AP Bug变化最小值</t>
-  </si>
-  <si>
-    <t>程序房间消耗2点行动点时，Bug变化随机下限（负数表示降低）</t>
-  </si>
-  <si>
-    <t>程序2AP Bug变化最大值</t>
-  </si>
-  <si>
-    <t>程序房间消耗2点行动点时，Bug变化随机上限（负数表示降低）</t>
-  </si>
-  <si>
-    <t>美术1AP画面变化最小值</t>
-  </si>
-  <si>
-    <t>美术房间消耗1点行动点时，画面变化随机下限</t>
-  </si>
-  <si>
-    <t>美术1AP画面变化最大值</t>
-  </si>
-  <si>
-    <t>美术房间消耗1点行动点时，画面变化随机上限</t>
-  </si>
-  <si>
-    <t>美术2AP画面变化最小值</t>
-  </si>
-  <si>
-    <t>美术房间消耗2点行动点时，画面变化随机下限</t>
-  </si>
-  <si>
-    <t>美术2AP画面变化最大值</t>
-  </si>
-  <si>
-    <t>美术房间消耗2点行动点时，画面变化随机上限</t>
-  </si>
-  <si>
-    <t>音效1AP氛围变化最小值</t>
-  </si>
-  <si>
-    <t>音效房间消耗1点行动点时，氛围变化随机下限</t>
-  </si>
-  <si>
-    <t>音效1AP氛围变化最大值</t>
-  </si>
-  <si>
-    <t>音效房间消耗1点行动点时，氛围变化随机上限</t>
-  </si>
-  <si>
-    <t>音效2AP氛围变化最小值</t>
-  </si>
-  <si>
-    <t>音效房间消耗2点行动点时，氛围变化随机下限</t>
-  </si>
-  <si>
-    <t>音效2AP氛围变化最大值</t>
-  </si>
-  <si>
-    <t>音效房间消耗2点行动点时，氛围变化随机上限</t>
-  </si>
-  <si>
-    <t>每次商店购买次数</t>
-  </si>
-  <si>
-    <t>每次进入商店时可购买Buff的次数</t>
-  </si>
-  <si>
-    <t>当前商店购买次数</t>
-  </si>
-  <si>
-    <t>当前商店阶段剩余可购买Buff的次数，进入商店时按每次商店购买次数重置</t>
-  </si>
-  <si>
-    <t>当前月第几周</t>
-  </si>
-  <si>
-    <t>只读流程镜像；用于配表条件判断，表示当前月内第几周，不允许通过事件或Buff修改</t>
-  </si>
-  <si>
-    <t>全局第几周</t>
-  </si>
-  <si>
-    <t>只读流程镜像；用于配表条件判断，表示从开局累计到当前的第几周，不允许通过事件或Buff修改</t>
-  </si>
-  <si>
-    <t>本周程序AP额外Bug变化</t>
-  </si>
-  <si>
-    <t>本周每消耗1点程序AP时额外应用的Bug变化；进入下一周自动清零</t>
-  </si>
-  <si>
-    <t>本周美术AP额外画面变化</t>
-  </si>
-  <si>
-    <t>本周每消耗1点美术AP时额外应用的画面变化；进入下一周自动清零</t>
-  </si>
-  <si>
-    <t>本周音频AP额外氛围变化</t>
-  </si>
-  <si>
-    <t>本周每消耗1点音频AP时额外应用的氛围变化；进入下一周自动清零</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1012,7 +1013,7 @@
         <v>38</v>
       </c>
       <c r="D17" s="3">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="E17" s="3" t="s">
         <v>39</v>
@@ -1027,10 +1028,10 @@
         <v>40</v>
       </c>
       <c r="D18" s="3">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>41</v>
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="70" customHeight="1" x14ac:dyDescent="0.25">
@@ -1039,13 +1040,13 @@
         <v>1007</v>
       </c>
       <c r="C19" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="D19" s="3">
+        <v>10</v>
+      </c>
+      <c r="E19" s="3" t="s">
         <v>42</v>
-      </c>
-      <c r="D19" s="3">
-        <v>0</v>
-      </c>
-      <c r="E19" s="3" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="70" customHeight="1" x14ac:dyDescent="0.25">
@@ -1054,13 +1055,13 @@
         <v>1028</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="s">
         <v>44</v>
-      </c>
-      <c r="D20" s="3">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1069,13 +1070,13 @@
         <v>1029</v>
       </c>
       <c r="C21" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="D21" s="3">
-        <v>0</v>
-      </c>
-      <c r="E21" s="3" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="22" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1084,13 +1085,13 @@
         <v>1030</v>
       </c>
       <c r="C22" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="s">
         <v>48</v>
-      </c>
-      <c r="D22" s="3">
-        <v>0</v>
-      </c>
-      <c r="E22" s="3" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1099,13 +1100,13 @@
         <v>1011</v>
       </c>
       <c r="C23" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="D23" s="3">
-        <v>0</v>
-      </c>
-      <c r="E23" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1114,13 +1115,13 @@
         <v>1012</v>
       </c>
       <c r="C24" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="3">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="s">
         <v>52</v>
-      </c>
-      <c r="D24" s="3">
-        <v>0</v>
-      </c>
-      <c r="E24" s="3" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1129,13 +1130,13 @@
         <v>1017</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D25" s="3">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="D25" s="3">
-        <v>0</v>
-      </c>
-      <c r="E25" s="3" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="26" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -1144,13 +1145,13 @@
         <v>1013</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="3">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3" t="s">
         <v>56</v>
-      </c>
-      <c r="D26" s="3">
-        <v>0</v>
-      </c>
-      <c r="E26" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="42" customHeight="1" x14ac:dyDescent="0.25">
@@ -1159,13 +1160,13 @@
         <v>1014</v>
       </c>
       <c r="C27" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="3">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3" t="s">
         <v>58</v>
-      </c>
-      <c r="D27" s="3">
-        <v>0</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="28" customHeight="1" x14ac:dyDescent="0.25">
@@ -1174,13 +1175,13 @@
         <v>1018</v>
       </c>
       <c r="C28" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D28" s="3">
+        <v>0</v>
+      </c>
+      <c r="E28" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="D28" s="3">
-        <v>0</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="56" customHeight="1" x14ac:dyDescent="0.25">
@@ -1189,13 +1190,13 @@
         <v>1015</v>
       </c>
       <c r="C29" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" s="3">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3" t="s">
         <v>62</v>
-      </c>
-      <c r="D29" s="3">
-        <v>0</v>
-      </c>
-      <c r="E29" s="3" t="s">
-        <v>63</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="70" customHeight="1" x14ac:dyDescent="0.25">
@@ -1204,13 +1205,13 @@
         <v>1016</v>
       </c>
       <c r="C30" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="3">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="D30" s="3">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="84" customHeight="1" x14ac:dyDescent="0.25">
@@ -1219,13 +1220,13 @@
         <v>1019</v>
       </c>
       <c r="C31" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="D31" s="3">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3" t="s">
         <v>66</v>
-      </c>
-      <c r="D31" s="3">
-        <v>0</v>
-      </c>
-      <c r="E31" s="3" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="32" spans="1:5" ht="56" x14ac:dyDescent="0.25">
@@ -1234,13 +1235,13 @@
         <v>1020</v>
       </c>
       <c r="C32" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="3">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="D32" s="3">
-        <v>0</v>
-      </c>
-      <c r="E32" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="33" spans="1:5" ht="56" x14ac:dyDescent="0.25">
@@ -1249,13 +1250,13 @@
         <v>1021</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="D33" s="3">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3" t="s">
         <v>70</v>
-      </c>
-      <c r="D33" s="3">
-        <v>0</v>
-      </c>
-      <c r="E33" s="3" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="34" spans="1:5" ht="42" x14ac:dyDescent="0.25">
@@ -1264,13 +1265,13 @@
         <v>1022</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D34" s="3">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>72</v>
-      </c>
-      <c r="D34" s="3">
-        <v>0</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="35" spans="1:5" ht="42" x14ac:dyDescent="0.25">
@@ -1279,13 +1280,13 @@
         <v>1023</v>
       </c>
       <c r="C35" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D35" s="3">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3" t="s">
         <v>74</v>
-      </c>
-      <c r="D35" s="3">
-        <v>0</v>
-      </c>
-      <c r="E35" s="3" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="28" x14ac:dyDescent="0.25">
@@ -1294,13 +1295,13 @@
         <v>1024</v>
       </c>
       <c r="C36" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D36" s="3">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="s">
         <v>76</v>
-      </c>
-      <c r="D36" s="3">
-        <v>0</v>
-      </c>
-      <c r="E36" s="3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:5" ht="56" x14ac:dyDescent="0.25">
@@ -1309,13 +1310,13 @@
         <v>1025</v>
       </c>
       <c r="C37" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="D37" s="3">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="s">
         <v>78</v>
-      </c>
-      <c r="D37" s="3">
-        <v>0</v>
-      </c>
-      <c r="E37" s="3" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="70" x14ac:dyDescent="0.25">
@@ -1324,13 +1325,13 @@
         <v>1026</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D38" s="3">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3" t="s">
         <v>80</v>
-      </c>
-      <c r="D38" s="3">
-        <v>0</v>
-      </c>
-      <c r="E38" s="3" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1338,13 +1339,13 @@
         <v>1031</v>
       </c>
       <c r="C39" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D39">
         <v>-4</v>
       </c>
       <c r="E39" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1352,13 +1353,13 @@
         <v>1032</v>
       </c>
       <c r="C40" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D40">
         <v>-2</v>
       </c>
       <c r="E40" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1366,13 +1367,13 @@
         <v>1033</v>
       </c>
       <c r="C41" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D41">
         <v>-9</v>
       </c>
       <c r="E41" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1380,13 +1381,13 @@
         <v>1034</v>
       </c>
       <c r="C42" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D42">
         <v>-6</v>
       </c>
       <c r="E42" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -1394,13 +1395,13 @@
         <v>1035</v>
       </c>
       <c r="C43" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D43">
         <v>4</v>
       </c>
       <c r="E43" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -1408,13 +1409,13 @@
         <v>1036</v>
       </c>
       <c r="C44" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D44">
         <v>6</v>
       </c>
       <c r="E44" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -1422,13 +1423,13 @@
         <v>1037</v>
       </c>
       <c r="C45" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D45">
         <v>10</v>
       </c>
       <c r="E45" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -1436,13 +1437,13 @@
         <v>1038</v>
       </c>
       <c r="C46" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D46">
         <v>13</v>
       </c>
       <c r="E46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
@@ -1450,13 +1451,13 @@
         <v>1039</v>
       </c>
       <c r="C47" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D47">
         <v>4</v>
       </c>
       <c r="E47" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -1464,13 +1465,13 @@
         <v>1040</v>
       </c>
       <c r="C48" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D48">
         <v>6</v>
       </c>
       <c r="E48" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="49" spans="2:5" x14ac:dyDescent="0.25">
@@ -1478,13 +1479,13 @@
         <v>1041</v>
       </c>
       <c r="C49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D49">
         <v>10</v>
       </c>
       <c r="E49" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="50" spans="2:5" x14ac:dyDescent="0.25">
@@ -1492,13 +1493,13 @@
         <v>1042</v>
       </c>
       <c r="C50" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D50">
         <v>13</v>
       </c>
       <c r="E50" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="2:5" x14ac:dyDescent="0.25">
@@ -1506,13 +1507,13 @@
         <v>1049</v>
       </c>
       <c r="C51" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D51">
         <v>2</v>
       </c>
       <c r="E51" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="52" spans="2:5" x14ac:dyDescent="0.25">
@@ -1520,13 +1521,13 @@
         <v>1050</v>
       </c>
       <c r="C52" t="s">
+        <v>107</v>
+      </c>
+      <c r="D52">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
         <v>108</v>
-      </c>
-      <c r="D52">
-        <v>0</v>
-      </c>
-      <c r="E52" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.25">
@@ -1534,13 +1535,13 @@
         <v>1051</v>
       </c>
       <c r="C53" t="s">
+        <v>109</v>
+      </c>
+      <c r="D53">
+        <v>0</v>
+      </c>
+      <c r="E53" t="s">
         <v>110</v>
-      </c>
-      <c r="D53">
-        <v>0</v>
-      </c>
-      <c r="E53" t="s">
-        <v>111</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.25">
@@ -1548,13 +1549,13 @@
         <v>1052</v>
       </c>
       <c r="C54" t="s">
+        <v>111</v>
+      </c>
+      <c r="D54">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
         <v>112</v>
-      </c>
-      <c r="D54">
-        <v>0</v>
-      </c>
-      <c r="E54" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.25">
@@ -1562,13 +1563,13 @@
         <v>1053</v>
       </c>
       <c r="C55" t="s">
+        <v>113</v>
+      </c>
+      <c r="D55">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
         <v>114</v>
-      </c>
-      <c r="D55">
-        <v>0</v>
-      </c>
-      <c r="E55" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.25">
@@ -1576,13 +1577,13 @@
         <v>1054</v>
       </c>
       <c r="C56" t="s">
+        <v>115</v>
+      </c>
+      <c r="D56">
+        <v>0</v>
+      </c>
+      <c r="E56" t="s">
         <v>116</v>
-      </c>
-      <c r="D56">
-        <v>0</v>
-      </c>
-      <c r="E56" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.25">
@@ -1590,13 +1591,13 @@
         <v>1055</v>
       </c>
       <c r="C57" t="s">
+        <v>117</v>
+      </c>
+      <c r="D57">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
         <v>118</v>
-      </c>
-      <c r="D57">
-        <v>0</v>
-      </c>
-      <c r="E57" t="s">
-        <v>119</v>
       </c>
     </row>
   </sheetData>

</xml_diff>